<commit_message>
Group materials with inline alternatives
</commit_message>
<xml_diff>
--- a/public/material-upload-template.xlsx
+++ b/public/material-upload-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上傳資料" sheetId="1" r:id="R01e0b269d9d74f6c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填寫說明" sheetId="2" r:id="R4d816f3c4bed478e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上傳資料" sheetId="1" r:id="R2767f8ad1ecf402d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填寫說明" sheetId="2" r:id="R1c457dbe3f9541d5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1054,7 +1054,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra9ae1aa72e324f69"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R866ed9cc0ef74e82"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1236,13 +1236,13 @@
         <x:v>分組</x:v>
       </x:c>
       <x:c r="B15" s="98" t="str">
-        <x:v>依 Ref Group、Ref Des，或料名＋規格＋Footprint 推斷。</x:v>
+        <x:v>有 Ref Group 時依 Ref Group＋料名；沒有時依模組＋料名分組。</x:v>
       </x:c>
       <x:c r="C15" s="98" t="str">
-        <x:v>同料固定填 Ref_tmp。</x:v>
+        <x:v>同料固定填 Ref_tmp；沒有群組時確保 Module 與 Name 一致。</x:v>
       </x:c>
       <x:c r="D15" s="99" t="str">
-        <x:v>不要只靠相似料名讓系統猜。</x:v>
+        <x:v>Ref Des 只代表電路位號，不作為替代料分組。</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="48" customHeight="1">

</xml_diff>